<commit_message>
Add rugby season-squad game: draft, subs, scoring, and admin tooling
Players draft one from each team (6 total, one designated kicker) once
before Round 1. The kicker scores for tries and every kick; the other
five score for tries only. Free substitutions (admin-tunable count) can
be made per team throughout the season; going beyond the free budget
costs points, as does a red card on any of the six. A differential
bonus rewards picking players few others hold, frozen at the moment
each player joins the squad.

Also: admin pages to manage rugby players/results/scoring-rules without
touching the spreadsheet, a new-season how-to guide, and a visual pass
bringing /rugby in line with the football site's pop-art look (it was
missing the .pop-art-theme class the CSS variables are actually scoped
to, which meant every colour was silently resolving to nothing).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/rugby-data.xlsx
+++ b/public/rugby-data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="350">
   <si>
     <t>Six Nations data sheet — how to fill this in</t>
   </si>
@@ -773,6 +773,243 @@
   </si>
   <si>
     <t>Max Spring</t>
+  </si>
+  <si>
+    <t>Trevor Davison</t>
+  </si>
+  <si>
+    <t>Bevan Rodd</t>
+  </si>
+  <si>
+    <t>Maro Itoje</t>
+  </si>
+  <si>
+    <t>Chandler Cunningham-South</t>
+  </si>
+  <si>
+    <t>Sam Underhill</t>
+  </si>
+  <si>
+    <t>Fraser Dingwall</t>
+  </si>
+  <si>
+    <t>Henry Arundell</t>
+  </si>
+  <si>
+    <t>Elliot Daly</t>
+  </si>
+  <si>
+    <t>Julien Marchand</t>
+  </si>
+  <si>
+    <t>Dorian Aldegheri</t>
+  </si>
+  <si>
+    <t>Uini Atonio</t>
+  </si>
+  <si>
+    <t>Cyril Baille</t>
+  </si>
+  <si>
+    <t>Jean-Baptiste Gros</t>
+  </si>
+  <si>
+    <t>Rodrigue Neti</t>
+  </si>
+  <si>
+    <t>Dany Priso</t>
+  </si>
+  <si>
+    <t>Thibaud Flament</t>
+  </si>
+  <si>
+    <t>Cameron Woki</t>
+  </si>
+  <si>
+    <t>Paul Boudehent</t>
+  </si>
+  <si>
+    <t>François Cros</t>
+  </si>
+  <si>
+    <t>Alexandre Fischer</t>
+  </si>
+  <si>
+    <t>Anthony Jelonch</t>
+  </si>
+  <si>
+    <t>Charles Ollivon</t>
+  </si>
+  <si>
+    <t>Thibault Daubagna</t>
+  </si>
+  <si>
+    <t>Antoine Dupont</t>
+  </si>
+  <si>
+    <t>Baptiste Serin</t>
+  </si>
+  <si>
+    <t>Ugo Seunes</t>
+  </si>
+  <si>
+    <t>Noah Nene</t>
+  </si>
+  <si>
+    <t>Louis Bielle-Biarrey</t>
+  </si>
+  <si>
+    <t>Gaël Dréan</t>
+  </si>
+  <si>
+    <t>Grégoire Arfeuil</t>
+  </si>
+  <si>
+    <t>Romain Buros</t>
+  </si>
+  <si>
+    <t>Thomas Ramos</t>
+  </si>
+  <si>
+    <t>Georges-Henri Colombe</t>
+  </si>
+  <si>
+    <t>Joshua Brennan</t>
+  </si>
+  <si>
+    <t>Jack Boyle</t>
+  </si>
+  <si>
+    <t>Michael Milne</t>
+  </si>
+  <si>
+    <t>Finlay Bealham</t>
+  </si>
+  <si>
+    <t>Thomas Ahern</t>
+  </si>
+  <si>
+    <t>Edwin Edogbo</t>
+  </si>
+  <si>
+    <t>Caelan Doris</t>
+  </si>
+  <si>
+    <t>Jack Crowley</t>
+  </si>
+  <si>
+    <t>Tom Farrell</t>
+  </si>
+  <si>
+    <t>James Lowe</t>
+  </si>
+  <si>
+    <t>Tommy O'Brien</t>
+  </si>
+  <si>
+    <t>Jude Postlethwaite</t>
+  </si>
+  <si>
+    <t>Giacomo Nicotera</t>
+  </si>
+  <si>
+    <t>Simone Ferrari</t>
+  </si>
+  <si>
+    <t>Alessandro Izekor</t>
+  </si>
+  <si>
+    <t>Samuele Locatelli</t>
+  </si>
+  <si>
+    <t>Manuel Zuliani</t>
+  </si>
+  <si>
+    <t>Martin Page-Relo</t>
+  </si>
+  <si>
+    <t>Damiano Mazza</t>
+  </si>
+  <si>
+    <t>Edoardo Todaro</t>
+  </si>
+  <si>
+    <t>Matt Gallagher</t>
+  </si>
+  <si>
+    <t>Giosuè Zilocchi</t>
+  </si>
+  <si>
+    <t>Dave Cherry</t>
+  </si>
+  <si>
+    <t>George Turner</t>
+  </si>
+  <si>
+    <t>Alex Craig</t>
+  </si>
+  <si>
+    <t>Grant Gilchrist</t>
+  </si>
+  <si>
+    <t>Jamie Ritchie</t>
+  </si>
+  <si>
+    <t>Adam Hastings</t>
+  </si>
+  <si>
+    <t>Huw Jones</t>
+  </si>
+  <si>
+    <t>Blair Kinghorn</t>
+  </si>
+  <si>
+    <t>Gus Warr</t>
+  </si>
+  <si>
+    <t>Liam Belcher</t>
+  </si>
+  <si>
+    <t>Keiron Assiratti</t>
+  </si>
+  <si>
+    <t>Tomas Francis</t>
+  </si>
+  <si>
+    <t>Archie Griffin</t>
+  </si>
+  <si>
+    <t>Dafydd Jenkins</t>
+  </si>
+  <si>
+    <t>Freddie Thomas</t>
+  </si>
+  <si>
+    <t>Olly Cracknell</t>
+  </si>
+  <si>
+    <t>Harri Deaves</t>
+  </si>
+  <si>
+    <t>Josh Macleod</t>
+  </si>
+  <si>
+    <t>Jarrod Evans</t>
+  </si>
+  <si>
+    <t>Louie Hennessey</t>
+  </si>
+  <si>
+    <t>Owen Watkin</t>
+  </si>
+  <si>
+    <t>Tom Rogers</t>
+  </si>
+  <si>
+    <t>Gabriel Hamer-Webb</t>
+  </si>
+  <si>
+    <t>Rhys Davies</t>
   </si>
   <si>
     <t>Round</t>
@@ -1410,13 +1647,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B400"/>
+  <dimension ref="A1:B297"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -3167,188 +3404,638 @@
         <v>251</v>
       </c>
     </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="267" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="270" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="271" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="272" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="274" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="275" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="276" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="277" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="278" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="279" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="280" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="281" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="283" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="284" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="285" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="286" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="287" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="288" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="332" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="333" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="334" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="335" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="336" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="337" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="338" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="339" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="340" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="341" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="342" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="343" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="344" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="345" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="346" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="347" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="348" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="349" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="350" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="351" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="352" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="353" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="354" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="355" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="356" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="357" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="358" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="359" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="360" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="361" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="362" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="363" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="364" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="365" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="366" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="367" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="368" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="369" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="370" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="371" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="372" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="373" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="374" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="375" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="376" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="377" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="378" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="379" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="380" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="381" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="382" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="383" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="384" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="385" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="386" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="387" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="388" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="389" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="390" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="391" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="392" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="393" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="394" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="395" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="396" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="397" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="398" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="399" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="400" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>29</v>
+      </c>
+      <c r="B219" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>29</v>
+      </c>
+      <c r="B220" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>29</v>
+      </c>
+      <c r="B221" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>29</v>
+      </c>
+      <c r="B222" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>29</v>
+      </c>
+      <c r="B223" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>29</v>
+      </c>
+      <c r="B224" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>29</v>
+      </c>
+      <c r="B225" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>29</v>
+      </c>
+      <c r="B226" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>209</v>
+      </c>
+      <c r="B227" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>209</v>
+      </c>
+      <c r="B228" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>209</v>
+      </c>
+      <c r="B229" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>209</v>
+      </c>
+      <c r="B230" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>209</v>
+      </c>
+      <c r="B231" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>209</v>
+      </c>
+      <c r="B232" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>209</v>
+      </c>
+      <c r="B233" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>209</v>
+      </c>
+      <c r="B234" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>209</v>
+      </c>
+      <c r="B235" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>209</v>
+      </c>
+      <c r="B236" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>209</v>
+      </c>
+      <c r="B237" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>209</v>
+      </c>
+      <c r="B238" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>209</v>
+      </c>
+      <c r="B239" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>209</v>
+      </c>
+      <c r="B240" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>209</v>
+      </c>
+      <c r="B241" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>209</v>
+      </c>
+      <c r="B242" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>209</v>
+      </c>
+      <c r="B243" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>209</v>
+      </c>
+      <c r="B244" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>209</v>
+      </c>
+      <c r="B245" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>209</v>
+      </c>
+      <c r="B246" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>209</v>
+      </c>
+      <c r="B247" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>209</v>
+      </c>
+      <c r="B248" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>209</v>
+      </c>
+      <c r="B249" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>209</v>
+      </c>
+      <c r="B250" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>209</v>
+      </c>
+      <c r="B251" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>209</v>
+      </c>
+      <c r="B252" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>67</v>
+      </c>
+      <c r="B253" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>67</v>
+      </c>
+      <c r="B254" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>67</v>
+      </c>
+      <c r="B255" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>67</v>
+      </c>
+      <c r="B256" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>67</v>
+      </c>
+      <c r="B257" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>67</v>
+      </c>
+      <c r="B258" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>67</v>
+      </c>
+      <c r="B259" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>67</v>
+      </c>
+      <c r="B260" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>67</v>
+      </c>
+      <c r="B261" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>67</v>
+      </c>
+      <c r="B262" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>67</v>
+      </c>
+      <c r="B263" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>141</v>
+      </c>
+      <c r="B264" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>141</v>
+      </c>
+      <c r="B265" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>141</v>
+      </c>
+      <c r="B266" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>141</v>
+      </c>
+      <c r="B267" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>141</v>
+      </c>
+      <c r="B268" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>141</v>
+      </c>
+      <c r="B269" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>141</v>
+      </c>
+      <c r="B270" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>141</v>
+      </c>
+      <c r="B271" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>141</v>
+      </c>
+      <c r="B272" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>141</v>
+      </c>
+      <c r="B273" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>104</v>
+      </c>
+      <c r="B274" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>104</v>
+      </c>
+      <c r="B275" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>104</v>
+      </c>
+      <c r="B276" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>104</v>
+      </c>
+      <c r="B277" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>104</v>
+      </c>
+      <c r="B278" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>104</v>
+      </c>
+      <c r="B279" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>104</v>
+      </c>
+      <c r="B280" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>104</v>
+      </c>
+      <c r="B281" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>104</v>
+      </c>
+      <c r="B282" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>175</v>
+      </c>
+      <c r="B283" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>175</v>
+      </c>
+      <c r="B284" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>175</v>
+      </c>
+      <c r="B285" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>175</v>
+      </c>
+      <c r="B286" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>175</v>
+      </c>
+      <c r="B287" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>175</v>
+      </c>
+      <c r="B288" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>175</v>
+      </c>
+      <c r="B289" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>175</v>
+      </c>
+      <c r="B290" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>175</v>
+      </c>
+      <c r="B291" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>175</v>
+      </c>
+      <c r="B292" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>175</v>
+      </c>
+      <c r="B293" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>175</v>
+      </c>
+      <c r="B294" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>175</v>
+      </c>
+      <c r="B295" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>175</v>
+      </c>
+      <c r="B296" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>175</v>
+      </c>
+      <c r="B297" t="s">
+        <v>330</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="A10:A400">
@@ -3359,7 +4046,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3378,34 +4065,34 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>252</v>
+        <v>331</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>253</v>
+        <v>332</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>254</v>
+        <v>333</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>255</v>
+        <v>334</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>256</v>
+        <v>335</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>257</v>
+        <v>336</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>258</v>
+        <v>337</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>259</v>
+        <v>338</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3419,7 +4106,7 @@
         <v>46423.84027777778</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3433,7 +4120,7 @@
         <v>46424.59027777778</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -3447,7 +4134,7 @@
         <v>46424.694444444445</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -3461,7 +4148,7 @@
         <v>46431.59027777778</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -3475,7 +4162,7 @@
         <v>46431.694444444445</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
@@ -3489,7 +4176,7 @@
         <v>46432.631944444445</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
@@ -3503,7 +4190,7 @@
         <v>46438.59027777778</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -3517,7 +4204,7 @@
         <v>46438.694444444445</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>3</v>
       </c>
@@ -3531,7 +4218,7 @@
         <v>46439.631944444445</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4</v>
       </c>
@@ -3545,7 +4232,7 @@
         <v>46451.84027777778</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>4</v>
       </c>
@@ -3559,7 +4246,7 @@
         <v>46452.59027777778</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
@@ -3573,7 +4260,7 @@
         <v>46452.694444444445</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
@@ -3587,7 +4274,7 @@
         <v>46459.59027777778</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>5</v>
       </c>
@@ -3601,7 +4288,7 @@
         <v>46459.694444444445</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5</v>
       </c>
@@ -3615,1156 +4302,1156 @@
         <v>46459.84027777778</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" s="5"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D18" s="5"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" s="5"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D20" s="5"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D21" s="5"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D22" s="5"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D23" s="5"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D24" s="5"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D25" s="5"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D26" s="5"/>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D27" s="5"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D28" s="5"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D29" s="5"/>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D30" s="5"/>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D31" s="5"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D32" s="5"/>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D33" s="5"/>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D34" s="5"/>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D35" s="5"/>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D36" s="5"/>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D37" s="5"/>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D40" s="5"/>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D41" s="5"/>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D42" s="5"/>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D43" s="5"/>
     </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D44" s="5"/>
     </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D45" s="5"/>
     </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D46" s="5"/>
     </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D47" s="5"/>
     </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D48" s="5"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D49" s="5"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D50" s="5"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D51" s="5"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D52" s="5"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D53" s="5"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D54" s="5"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D55" s="5"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D56" s="5"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D57" s="5"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D58" s="5"/>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D59" s="5"/>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D60" s="5"/>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D61" s="5"/>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D62" s="5"/>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D63" s="5"/>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D64" s="5"/>
     </row>
-    <row r="65" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D65" s="5"/>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D66" s="5"/>
     </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D67" s="5"/>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D68" s="5"/>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D69" s="5"/>
     </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D70" s="5"/>
     </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D71" s="5"/>
     </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D72" s="5"/>
     </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D73" s="5"/>
     </row>
-    <row r="74" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D74" s="5"/>
     </row>
-    <row r="75" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D75" s="5"/>
     </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D76" s="5"/>
     </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D77" s="5"/>
     </row>
-    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D78" s="5"/>
     </row>
-    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D79" s="5"/>
     </row>
-    <row r="80" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D80" s="5"/>
     </row>
-    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D81" s="5"/>
     </row>
-    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D82" s="5"/>
     </row>
-    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D83" s="5"/>
     </row>
-    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D84" s="5"/>
     </row>
-    <row r="85" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D85" s="5"/>
     </row>
-    <row r="86" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D86" s="5"/>
     </row>
-    <row r="87" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D87" s="5"/>
     </row>
-    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D88" s="5"/>
     </row>
-    <row r="89" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D89" s="5"/>
     </row>
-    <row r="90" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D90" s="5"/>
     </row>
-    <row r="91" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D91" s="5"/>
     </row>
-    <row r="92" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D92" s="5"/>
     </row>
-    <row r="93" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D93" s="5"/>
     </row>
-    <row r="94" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D94" s="5"/>
     </row>
-    <row r="95" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D95" s="5"/>
     </row>
-    <row r="96" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D96" s="5"/>
     </row>
-    <row r="97" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D97" s="5"/>
     </row>
-    <row r="98" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D98" s="5"/>
     </row>
-    <row r="99" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D99" s="5"/>
     </row>
-    <row r="100" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D100" s="5"/>
     </row>
-    <row r="101" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D101" s="5"/>
     </row>
-    <row r="102" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D102" s="5"/>
     </row>
-    <row r="103" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D103" s="5"/>
     </row>
-    <row r="104" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D104" s="5"/>
     </row>
-    <row r="105" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D105" s="5"/>
     </row>
-    <row r="106" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D106" s="5"/>
     </row>
-    <row r="107" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D107" s="5"/>
     </row>
-    <row r="108" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D108" s="5"/>
     </row>
-    <row r="109" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D109" s="5"/>
     </row>
-    <row r="110" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D110" s="5"/>
     </row>
-    <row r="111" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D111" s="5"/>
     </row>
-    <row r="112" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D112" s="5"/>
     </row>
-    <row r="113" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D113" s="5"/>
     </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D114" s="5"/>
     </row>
-    <row r="115" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D115" s="5"/>
     </row>
-    <row r="116" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D116" s="5"/>
     </row>
-    <row r="117" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D117" s="5"/>
     </row>
-    <row r="118" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D118" s="5"/>
     </row>
-    <row r="119" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D119" s="5"/>
     </row>
-    <row r="120" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D120" s="5"/>
     </row>
-    <row r="121" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D121" s="5"/>
     </row>
-    <row r="122" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D122" s="5"/>
     </row>
-    <row r="123" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D123" s="5"/>
     </row>
-    <row r="124" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D124" s="5"/>
     </row>
-    <row r="125" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D125" s="5"/>
     </row>
-    <row r="126" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D126" s="5"/>
     </row>
-    <row r="127" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D127" s="5"/>
     </row>
-    <row r="128" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D128" s="5"/>
     </row>
-    <row r="129" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D129" s="5"/>
     </row>
-    <row r="130" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D130" s="5"/>
     </row>
-    <row r="131" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D131" s="5"/>
     </row>
-    <row r="132" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D132" s="5"/>
     </row>
-    <row r="133" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D133" s="5"/>
     </row>
-    <row r="134" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D134" s="5"/>
     </row>
-    <row r="135" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D135" s="5"/>
     </row>
-    <row r="136" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D136" s="5"/>
     </row>
-    <row r="137" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D137" s="5"/>
     </row>
-    <row r="138" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D138" s="5"/>
     </row>
-    <row r="139" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D139" s="5"/>
     </row>
-    <row r="140" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D140" s="5"/>
     </row>
-    <row r="141" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D141" s="5"/>
     </row>
-    <row r="142" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D142" s="5"/>
     </row>
-    <row r="143" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D143" s="5"/>
     </row>
-    <row r="144" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D144" s="5"/>
     </row>
-    <row r="145" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D145" s="5"/>
     </row>
-    <row r="146" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D146" s="5"/>
     </row>
-    <row r="147" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D147" s="5"/>
     </row>
-    <row r="148" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D148" s="5"/>
     </row>
-    <row r="149" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D149" s="5"/>
     </row>
-    <row r="150" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D150" s="5"/>
     </row>
-    <row r="151" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D151" s="5"/>
     </row>
-    <row r="152" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D152" s="5"/>
     </row>
-    <row r="153" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="153" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D153" s="5"/>
     </row>
-    <row r="154" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="154" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D154" s="5"/>
     </row>
-    <row r="155" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="155" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D155" s="5"/>
     </row>
-    <row r="156" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="156" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D156" s="5"/>
     </row>
-    <row r="157" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="157" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D157" s="5"/>
     </row>
-    <row r="158" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="158" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D158" s="5"/>
     </row>
-    <row r="159" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="159" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D159" s="5"/>
     </row>
-    <row r="160" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D160" s="5"/>
     </row>
-    <row r="161" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="161" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D161" s="5"/>
     </row>
-    <row r="162" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="162" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D162" s="5"/>
     </row>
-    <row r="163" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D163" s="5"/>
     </row>
-    <row r="164" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D164" s="5"/>
     </row>
-    <row r="165" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D165" s="5"/>
     </row>
-    <row r="166" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D166" s="5"/>
     </row>
-    <row r="167" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D167" s="5"/>
     </row>
-    <row r="168" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D168" s="5"/>
     </row>
-    <row r="169" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D169" s="5"/>
     </row>
-    <row r="170" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D170" s="5"/>
     </row>
-    <row r="171" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D171" s="5"/>
     </row>
-    <row r="172" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D172" s="5"/>
     </row>
-    <row r="173" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D173" s="5"/>
     </row>
-    <row r="174" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D174" s="5"/>
     </row>
-    <row r="175" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D175" s="5"/>
     </row>
-    <row r="176" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D176" s="5"/>
     </row>
-    <row r="177" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D177" s="5"/>
     </row>
-    <row r="178" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D178" s="5"/>
     </row>
-    <row r="179" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D179" s="5"/>
     </row>
-    <row r="180" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="180" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D180" s="5"/>
     </row>
-    <row r="181" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="181" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D181" s="5"/>
     </row>
-    <row r="182" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="182" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D182" s="5"/>
     </row>
-    <row r="183" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D183" s="5"/>
     </row>
-    <row r="184" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="184" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D184" s="5"/>
     </row>
-    <row r="185" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="185" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D185" s="5"/>
     </row>
-    <row r="186" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="186" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D186" s="5"/>
     </row>
-    <row r="187" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="187" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D187" s="5"/>
     </row>
-    <row r="188" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="188" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D188" s="5"/>
     </row>
-    <row r="189" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="189" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D189" s="5"/>
     </row>
-    <row r="190" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="190" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D190" s="5"/>
     </row>
-    <row r="191" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="191" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D191" s="5"/>
     </row>
-    <row r="192" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="192" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D192" s="5"/>
     </row>
-    <row r="193" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="193" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D193" s="5"/>
     </row>
-    <row r="194" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="194" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D194" s="5"/>
     </row>
-    <row r="195" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="195" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D195" s="5"/>
     </row>
-    <row r="196" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="196" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D196" s="5"/>
     </row>
-    <row r="197" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="197" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D197" s="5"/>
     </row>
-    <row r="198" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="198" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D198" s="5"/>
     </row>
-    <row r="199" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="199" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D199" s="5"/>
     </row>
-    <row r="200" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="200" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D200" s="5"/>
     </row>
-    <row r="201" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="201" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D201" s="5"/>
     </row>
-    <row r="202" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="202" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D202" s="5"/>
     </row>
-    <row r="203" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="203" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D203" s="5"/>
     </row>
-    <row r="204" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="204" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D204" s="5"/>
     </row>
-    <row r="205" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="205" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D205" s="5"/>
     </row>
-    <row r="206" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="206" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D206" s="5"/>
     </row>
-    <row r="207" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="207" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D207" s="5"/>
     </row>
-    <row r="208" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="208" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D208" s="5"/>
     </row>
-    <row r="209" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="209" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D209" s="5"/>
     </row>
-    <row r="210" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="210" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D210" s="5"/>
     </row>
-    <row r="211" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="211" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D211" s="5"/>
     </row>
-    <row r="212" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="212" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D212" s="5"/>
     </row>
-    <row r="213" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="213" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D213" s="5"/>
     </row>
-    <row r="214" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="214" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D214" s="5"/>
     </row>
-    <row r="215" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="215" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D215" s="5"/>
     </row>
-    <row r="216" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="216" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D216" s="5"/>
     </row>
-    <row r="217" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="217" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D217" s="5"/>
     </row>
-    <row r="218" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="218" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D218" s="5"/>
     </row>
-    <row r="219" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="219" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D219" s="5"/>
     </row>
-    <row r="220" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="220" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D220" s="5"/>
     </row>
-    <row r="221" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="221" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D221" s="5"/>
     </row>
-    <row r="222" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="222" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D222" s="5"/>
     </row>
-    <row r="223" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="223" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D223" s="5"/>
     </row>
-    <row r="224" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="224" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D224" s="5"/>
     </row>
-    <row r="225" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D225" s="5"/>
     </row>
-    <row r="226" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D226" s="5"/>
     </row>
-    <row r="227" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D227" s="5"/>
     </row>
-    <row r="228" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D228" s="5"/>
     </row>
-    <row r="229" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="229" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D229" s="5"/>
     </row>
-    <row r="230" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="230" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D230" s="5"/>
     </row>
-    <row r="231" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="231" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D231" s="5"/>
     </row>
-    <row r="232" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="232" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D232" s="5"/>
     </row>
-    <row r="233" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="233" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D233" s="5"/>
     </row>
-    <row r="234" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="234" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D234" s="5"/>
     </row>
-    <row r="235" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="235" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D235" s="5"/>
     </row>
-    <row r="236" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="236" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D236" s="5"/>
     </row>
-    <row r="237" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="237" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D237" s="5"/>
     </row>
-    <row r="238" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="238" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D238" s="5"/>
     </row>
-    <row r="239" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="239" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D239" s="5"/>
     </row>
-    <row r="240" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="240" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D240" s="5"/>
     </row>
-    <row r="241" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="241" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D241" s="5"/>
     </row>
-    <row r="242" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="242" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D242" s="5"/>
     </row>
-    <row r="243" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="243" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D243" s="5"/>
     </row>
-    <row r="244" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="244" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D244" s="5"/>
     </row>
-    <row r="245" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="245" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D245" s="5"/>
     </row>
-    <row r="246" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="246" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D246" s="5"/>
     </row>
-    <row r="247" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="247" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D247" s="5"/>
     </row>
-    <row r="248" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="248" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D248" s="5"/>
     </row>
-    <row r="249" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="249" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D249" s="5"/>
     </row>
-    <row r="250" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="250" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D250" s="5"/>
     </row>
-    <row r="251" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="251" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D251" s="5"/>
     </row>
-    <row r="252" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="252" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D252" s="5"/>
     </row>
-    <row r="253" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="253" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D253" s="5"/>
     </row>
-    <row r="254" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="254" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D254" s="5"/>
     </row>
-    <row r="255" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="255" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D255" s="5"/>
     </row>
-    <row r="256" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="256" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D256" s="5"/>
     </row>
-    <row r="257" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="257" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D257" s="5"/>
     </row>
-    <row r="258" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="258" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D258" s="5"/>
     </row>
-    <row r="259" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="259" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D259" s="5"/>
     </row>
-    <row r="260" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="260" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D260" s="5"/>
     </row>
-    <row r="261" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="261" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D261" s="5"/>
     </row>
-    <row r="262" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="262" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D262" s="5"/>
     </row>
-    <row r="263" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="263" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D263" s="5"/>
     </row>
-    <row r="264" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="264" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D264" s="5"/>
     </row>
-    <row r="265" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="265" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D265" s="5"/>
     </row>
-    <row r="266" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="266" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D266" s="5"/>
     </row>
-    <row r="267" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="267" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D267" s="5"/>
     </row>
-    <row r="268" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="268" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D268" s="5"/>
     </row>
-    <row r="269" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="269" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D269" s="5"/>
     </row>
-    <row r="270" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="270" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D270" s="5"/>
     </row>
-    <row r="271" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="271" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D271" s="5"/>
     </row>
-    <row r="272" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="272" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D272" s="5"/>
     </row>
-    <row r="273" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="273" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D273" s="5"/>
     </row>
-    <row r="274" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D274" s="5"/>
     </row>
-    <row r="275" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="275" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D275" s="5"/>
     </row>
-    <row r="276" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D276" s="5"/>
     </row>
-    <row r="277" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D277" s="5"/>
     </row>
-    <row r="278" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D278" s="5"/>
     </row>
-    <row r="279" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D279" s="5"/>
     </row>
-    <row r="280" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="280" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D280" s="5"/>
     </row>
-    <row r="281" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="281" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D281" s="5"/>
     </row>
-    <row r="282" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D282" s="5"/>
     </row>
-    <row r="283" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D283" s="5"/>
     </row>
-    <row r="284" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D284" s="5"/>
     </row>
-    <row r="285" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D285" s="5"/>
     </row>
-    <row r="286" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D286" s="5"/>
     </row>
-    <row r="287" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D287" s="5"/>
     </row>
-    <row r="288" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D288" s="5"/>
     </row>
-    <row r="289" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="289" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D289" s="5"/>
     </row>
-    <row r="290" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="290" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D290" s="5"/>
     </row>
-    <row r="291" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="291" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D291" s="5"/>
     </row>
-    <row r="292" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D292" s="5"/>
     </row>
-    <row r="293" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D293" s="5"/>
     </row>
-    <row r="294" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="294" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D294" s="5"/>
     </row>
-    <row r="295" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="295" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D295" s="5"/>
     </row>
-    <row r="296" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="296" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D296" s="5"/>
     </row>
-    <row r="297" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="297" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D297" s="5"/>
     </row>
-    <row r="298" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="298" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D298" s="5"/>
     </row>
-    <row r="299" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="299" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D299" s="5"/>
     </row>
-    <row r="300" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="300" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D300" s="5"/>
     </row>
-    <row r="301" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="301" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D301" s="5"/>
     </row>
-    <row r="302" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="302" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D302" s="5"/>
     </row>
-    <row r="303" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="303" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D303" s="5"/>
     </row>
-    <row r="304" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="304" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D304" s="5"/>
     </row>
-    <row r="305" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="305" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D305" s="5"/>
     </row>
-    <row r="306" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="306" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D306" s="5"/>
     </row>
-    <row r="307" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="307" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D307" s="5"/>
     </row>
-    <row r="308" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="308" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D308" s="5"/>
     </row>
-    <row r="309" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="309" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D309" s="5"/>
     </row>
-    <row r="310" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="310" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D310" s="5"/>
     </row>
-    <row r="311" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="311" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D311" s="5"/>
     </row>
-    <row r="312" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="312" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D312" s="5"/>
     </row>
-    <row r="313" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="313" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D313" s="5"/>
     </row>
-    <row r="314" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="314" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D314" s="5"/>
     </row>
-    <row r="315" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="315" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D315" s="5"/>
     </row>
-    <row r="316" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="316" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D316" s="5"/>
     </row>
-    <row r="317" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="317" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D317" s="5"/>
     </row>
-    <row r="318" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="318" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D318" s="5"/>
     </row>
-    <row r="319" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="319" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D319" s="5"/>
     </row>
-    <row r="320" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="320" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D320" s="5"/>
     </row>
-    <row r="321" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="321" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D321" s="5"/>
     </row>
-    <row r="322" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="322" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D322" s="5"/>
     </row>
-    <row r="323" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="323" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D323" s="5"/>
     </row>
-    <row r="324" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="324" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D324" s="5"/>
     </row>
-    <row r="325" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="325" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D325" s="5"/>
     </row>
-    <row r="326" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="326" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D326" s="5"/>
     </row>
-    <row r="327" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="327" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D327" s="5"/>
     </row>
-    <row r="328" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="328" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D328" s="5"/>
     </row>
-    <row r="329" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="329" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D329" s="5"/>
     </row>
-    <row r="330" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="330" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D330" s="5"/>
     </row>
-    <row r="331" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="331" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D331" s="5"/>
     </row>
-    <row r="332" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="332" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D332" s="5"/>
     </row>
-    <row r="333" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="333" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D333" s="5"/>
     </row>
-    <row r="334" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="334" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D334" s="5"/>
     </row>
-    <row r="335" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="335" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D335" s="5"/>
     </row>
-    <row r="336" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="336" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D336" s="5"/>
     </row>
-    <row r="337" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="337" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D337" s="5"/>
     </row>
-    <row r="338" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="338" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D338" s="5"/>
     </row>
-    <row r="339" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="339" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D339" s="5"/>
     </row>
-    <row r="340" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="340" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D340" s="5"/>
     </row>
-    <row r="341" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="341" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D341" s="5"/>
     </row>
-    <row r="342" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="342" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D342" s="5"/>
     </row>
-    <row r="343" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="343" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D343" s="5"/>
     </row>
-    <row r="344" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="344" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D344" s="5"/>
     </row>
-    <row r="345" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="345" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D345" s="5"/>
     </row>
-    <row r="346" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="346" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D346" s="5"/>
     </row>
-    <row r="347" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="347" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D347" s="5"/>
     </row>
-    <row r="348" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="348" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D348" s="5"/>
     </row>
-    <row r="349" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="349" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D349" s="5"/>
     </row>
-    <row r="350" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="350" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D350" s="5"/>
     </row>
-    <row r="351" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="351" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D351" s="5"/>
     </row>
-    <row r="352" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="352" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D352" s="5"/>
     </row>
-    <row r="353" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="353" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D353" s="5"/>
     </row>
-    <row r="354" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="354" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D354" s="5"/>
     </row>
-    <row r="355" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="355" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D355" s="5"/>
     </row>
-    <row r="356" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="356" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D356" s="5"/>
     </row>
-    <row r="357" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="357" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D357" s="5"/>
     </row>
-    <row r="358" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="358" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D358" s="5"/>
     </row>
-    <row r="359" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="359" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D359" s="5"/>
     </row>
-    <row r="360" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="360" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D360" s="5"/>
     </row>
-    <row r="361" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="361" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D361" s="5"/>
     </row>
-    <row r="362" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="362" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D362" s="5"/>
     </row>
-    <row r="363" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="363" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D363" s="5"/>
     </row>
-    <row r="364" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="364" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D364" s="5"/>
     </row>
-    <row r="365" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="365" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D365" s="5"/>
     </row>
-    <row r="366" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="366" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D366" s="5"/>
     </row>
-    <row r="367" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="367" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D367" s="5"/>
     </row>
-    <row r="368" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="368" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D368" s="5"/>
     </row>
-    <row r="369" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="369" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D369" s="5"/>
     </row>
-    <row r="370" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="370" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D370" s="5"/>
     </row>
-    <row r="371" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="371" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D371" s="5"/>
     </row>
-    <row r="372" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="372" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D372" s="5"/>
     </row>
-    <row r="373" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="373" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D373" s="5"/>
     </row>
-    <row r="374" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="374" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D374" s="5"/>
     </row>
-    <row r="375" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="375" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D375" s="5"/>
     </row>
-    <row r="376" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="376" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D376" s="5"/>
     </row>
-    <row r="377" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="377" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D377" s="5"/>
     </row>
-    <row r="378" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="378" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D378" s="5"/>
     </row>
-    <row r="379" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="379" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D379" s="5"/>
     </row>
-    <row r="380" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="380" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D380" s="5"/>
     </row>
-    <row r="381" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="381" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D381" s="5"/>
     </row>
-    <row r="382" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="382" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D382" s="5"/>
     </row>
-    <row r="383" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="383" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D383" s="5"/>
     </row>
-    <row r="384" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="384" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D384" s="5"/>
     </row>
-    <row r="385" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="385" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D385" s="5"/>
     </row>
-    <row r="386" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="386" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D386" s="5"/>
     </row>
-    <row r="387" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="387" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D387" s="5"/>
     </row>
-    <row r="388" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="388" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D388" s="5"/>
     </row>
-    <row r="389" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="389" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D389" s="5"/>
     </row>
-    <row r="390" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="390" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D390" s="5"/>
     </row>
-    <row r="391" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="391" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D391" s="5"/>
     </row>
-    <row r="392" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="392" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D392" s="5"/>
     </row>
-    <row r="393" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="393" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D393" s="5"/>
     </row>
-    <row r="394" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="394" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D394" s="5"/>
     </row>
-    <row r="395" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="395" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D395" s="5"/>
     </row>
-    <row r="396" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="396" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D396" s="5"/>
     </row>
-    <row r="397" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="397" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D397" s="5"/>
     </row>
-    <row r="398" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="398" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D398" s="5"/>
     </row>
-    <row r="399" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="399" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D399" s="5"/>
     </row>
-    <row r="400" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="400" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D400" s="5"/>
     </row>
   </sheetData>
@@ -4789,7 +5476,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4804,54 +5491,54 @@
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>261</v>
+        <v>340</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>262</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>263</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>264</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>265</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>266</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>267</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>269</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>270</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>